<commit_message>
Calculation is done, by changing the line 120 where the diff is using diff = expeced - final_credit. THis makes the calculation correct for now. will need to update with another thing such as minigames. for the time window where it will capture the total win and calculation into the regular games.
</commit_message>
<xml_diff>
--- a/Slot_result.xlsx
+++ b/Slot_result.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,20 +442,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Expected BalanceActual Balance</t>
+          <t>Expected Balance</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Actual Balance</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Difference</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
@@ -466,7 +471,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>100</v>
@@ -475,13 +480,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>-25</v>
+        <v>-100</v>
       </c>
       <c r="F2" t="n">
-        <v>4348475</v>
+        <v>4447122</v>
       </c>
       <c r="G2" t="n">
-        <v>4348500</v>
+        <v>-4447222</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -489,7 +494,7 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>46083.66508062097</v>
+        <v>46083.72264555664</v>
       </c>
     </row>
     <row r="3">
@@ -497,7 +502,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4348475</v>
+        <v>4447122</v>
       </c>
       <c r="C3" t="n">
         <v>100</v>
@@ -506,21 +511,21 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4348375</v>
+        <v>4447022</v>
       </c>
       <c r="F3" t="n">
-        <v>4348475</v>
+        <v>4447022</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>46083.66549963505</v>
+        <v>46083.72271831999</v>
       </c>
     </row>
     <row r="4">
@@ -528,30 +533,30 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4348475</v>
+        <v>4447022</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4348423</v>
+        <v>4446922</v>
       </c>
       <c r="F4" t="n">
-        <v>4348375</v>
+        <v>4446922</v>
       </c>
       <c r="G4" t="n">
-        <v>-48</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>46083.66566031661</v>
+        <v>46083.72277333462</v>
       </c>
     </row>
     <row r="5">
@@ -559,154 +564,30 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>4348375</v>
+        <v>4446922</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="E5" t="n">
-        <v>4348435</v>
+        <v>4447122</v>
       </c>
       <c r="F5" t="n">
-        <v>4348535</v>
+        <v>4447122</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>46083.66571468035</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>4348535</v>
-      </c>
-      <c r="C6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" t="n">
-        <v>16</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4348451</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4348435</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-16</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Incorrect</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>46083.66584317708</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>4348435</v>
-      </c>
-      <c r="C7" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" t="n">
-        <v>56</v>
-      </c>
-      <c r="E7" t="n">
-        <v>4348391</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4348491</v>
-      </c>
-      <c r="G7" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Incorrect</t>
-        </is>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>46083.66589824016</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>4348491</v>
-      </c>
-      <c r="C8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" t="n">
-        <v>158</v>
-      </c>
-      <c r="E8" t="n">
-        <v>4348549</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4348391</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-158</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Incorrect</t>
-        </is>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>46083.66609685222</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>4348391</v>
-      </c>
-      <c r="C9" t="n">
-        <v>100</v>
-      </c>
-      <c r="D9" t="n">
-        <v>528</v>
-      </c>
-      <c r="E9" t="n">
-        <v>4348819</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4348919</v>
-      </c>
-      <c r="G9" t="n">
-        <v>100</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Incorrect</t>
-        </is>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>46083.6661698186</v>
+        <v>46083.72286380359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculation work is done for the main game. Now need to improve with the minigame, first is the heng ong huat one. Next is the head or tail game
</commit_message>
<xml_diff>
--- a/Slot_result.xlsx
+++ b/Slot_result.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,7 +471,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>202518</v>
       </c>
       <c r="C2" t="n">
         <v>100</v>
@@ -480,13 +480,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>-100</v>
+        <v>202418</v>
       </c>
       <c r="F2" t="n">
-        <v>4447122</v>
+        <v>4542799</v>
       </c>
       <c r="G2" t="n">
-        <v>-4447222</v>
+        <v>-4340381</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>46083.72264555664</v>
+        <v>46084.43354696759</v>
       </c>
     </row>
     <row r="3">
@@ -502,7 +502,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4447122</v>
+        <v>4542799</v>
       </c>
       <c r="C3" t="n">
         <v>100</v>
@@ -511,10 +511,10 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4447022</v>
+        <v>4542699</v>
       </c>
       <c r="F3" t="n">
-        <v>4447022</v>
+        <v>4542699</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>46083.72271831999</v>
+        <v>46084.4336024537</v>
       </c>
     </row>
     <row r="4">
@@ -533,7 +533,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4447022</v>
+        <v>4542699</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
@@ -542,10 +542,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4446922</v>
+        <v>4542599</v>
       </c>
       <c r="F4" t="n">
-        <v>4446922</v>
+        <v>4542599</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>46083.72277333462</v>
+        <v>46084.43366769676</v>
       </c>
     </row>
     <row r="5">
@@ -564,19 +564,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>4446922</v>
+        <v>4542599</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>4447122</v>
+        <v>4542499</v>
       </c>
       <c r="F5" t="n">
-        <v>4447122</v>
+        <v>4542499</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -587,7 +587,317 @@
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>46083.72286380359</v>
+        <v>46084.43372659722</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>4542499</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4542399</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4542399</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>46084.43378716435</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>4542399</v>
+      </c>
+      <c r="C7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4542299</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4542787</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-488</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>46084.43385892361</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>202518</v>
+      </c>
+      <c r="C8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" t="n">
+        <v>144</v>
+      </c>
+      <c r="E8" t="n">
+        <v>202562</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4542831</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-4340269</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>46084.43417752582</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4542831</v>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" t="n">
+        <v>144</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4542875</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4542868</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>46084.43422598884</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" t="n">
+        <v>33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-60</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4542731</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-4542791</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>46084.43428504332</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4542731</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>90</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4542721</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4542821</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-100</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>46084.43433967098</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4542821</v>
+      </c>
+      <c r="C12" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4542721</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4542721</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>46084.43447571812</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4542721</v>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="n">
+        <v>180</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4542801</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4542801</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>46084.43460465053</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4542801</v>
+      </c>
+      <c r="C14" t="n">
+        <v>100</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4542701</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4542701</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>46084.43470820727</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4542701</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>144</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4542745</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4542745</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>46084.43480476935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Function of autoclicker implemented
</commit_message>
<xml_diff>
--- a/Slot_result.xlsx
+++ b/Slot_result.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,40 +427,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Prev Balance</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Bet</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total Win</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected Balance</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Actual Balance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
@@ -470,155 +475,180 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
-        <v>9202518</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E2" t="n">
-        <v>9202268</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>4613779</v>
+        <v>-200</v>
       </c>
       <c r="G2" t="n">
-        <v>4588489</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>4584164</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-4584364</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Incorrect</t>
         </is>
       </c>
-      <c r="I2" s="1" t="n">
-        <v>46084.60565237269</v>
+      <c r="J2" s="1" t="n">
+        <v>46084.69231315972</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
-        <v>4613779</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>250</v>
+        <v>4584164</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E3" t="n">
-        <v>4613529</v>
+        <v>2176</v>
       </c>
       <c r="F3" t="n">
-        <v>4613529</v>
+        <v>4586140</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>46084.60593363426</v>
+        <v>4584164</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1976</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>46084.69252571759</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>4613529</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jackpot</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>250</v>
+        <v>4584164</v>
       </c>
       <c r="D4" t="n">
-        <v>1785</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4615064</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
-        <v>4615064</v>
+        <v>4584172</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>46084.6061349537</v>
+      <c r="H4" t="n">
+        <v>4584172</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>46084.6928231713</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
-        <v>9202518</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E5" t="n">
-        <v>9202518</v>
+        <v>3172</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>2972</v>
       </c>
       <c r="G5" t="n">
-        <v>9202518</v>
-      </c>
-      <c r="H5" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2972</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Incorrect</t>
         </is>
       </c>
-      <c r="I5" s="1" t="n">
-        <v>46084.60917446759</v>
+      <c r="J5" s="1" t="n">
+        <v>46084.6928857176</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="n">
-        <v>4615064</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E6" t="n">
-        <v>4614814</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>4614814</v>
+        <v>-200</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>46084.60930747478</v>
+        <v>4587136</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-4587336</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>46084.69295581018</v>
       </c>
     </row>
     <row r="7">
@@ -626,22 +656,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>4614814</v>
+        <v>202518</v>
       </c>
       <c r="C7" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D7" t="n">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E7" t="n">
-        <v>4614704</v>
+        <v>202450</v>
       </c>
       <c r="F7" t="n">
-        <v>4614564</v>
+        <v>4587068</v>
       </c>
       <c r="G7" t="n">
-        <v>140</v>
+        <v>-4384618</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -649,7 +679,7 @@
         </is>
       </c>
       <c r="I7" s="1" t="n">
-        <v>46084.60936990834</v>
+        <v>46084.70384810185</v>
       </c>
     </row>
     <row r="8">
@@ -657,30 +687,30 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>4614564</v>
+        <v>4587068</v>
       </c>
       <c r="C8" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D8" t="n">
-        <v>560</v>
+        <v>240</v>
       </c>
       <c r="E8" t="n">
-        <v>4614874</v>
+        <v>4587108</v>
       </c>
       <c r="F8" t="n">
-        <v>4615124</v>
+        <v>4587108</v>
       </c>
       <c r="G8" t="n">
-        <v>-250</v>
+        <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I8" s="1" t="n">
-        <v>46084.60942412478</v>
+        <v>46084.70394574074</v>
       </c>
     </row>
     <row r="9">
@@ -688,22 +718,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>4615124</v>
+        <v>4587108</v>
       </c>
       <c r="C9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D9" t="n">
-        <v>1120</v>
+        <v>60</v>
       </c>
       <c r="E9" t="n">
-        <v>4615994</v>
+        <v>4586968</v>
       </c>
       <c r="F9" t="n">
-        <v>4615684</v>
+        <v>4586908</v>
       </c>
       <c r="G9" t="n">
-        <v>310</v>
+        <v>60</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -711,7 +741,689 @@
         </is>
       </c>
       <c r="I9" s="1" t="n">
-        <v>46084.60977122879</v>
+        <v>46084.70400822916</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4586908</v>
+      </c>
+      <c r="C10" t="n">
+        <v>200</v>
+      </c>
+      <c r="D10" t="n">
+        <v>240</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4586948</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4587148</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-200</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>46084.70406305556</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4587148</v>
+      </c>
+      <c r="C11" t="n">
+        <v>200</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4586948</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4586948</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>46084.70418261574</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4586948</v>
+      </c>
+      <c r="C12" t="n">
+        <v>200</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4586748</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4586748</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>46084.70427739583</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4586748</v>
+      </c>
+      <c r="C13" t="n">
+        <v>200</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4586548</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4586828</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-280</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>46084.70436921297</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>4586828</v>
+      </c>
+      <c r="C14" t="n">
+        <v>200</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4586628</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4586628</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>46084.70454583333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>4586628</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4586528</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4586716</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-188</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>46084.70467278935</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>4586716</v>
+      </c>
+      <c r="C16" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4586616</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4586808</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-192</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>46084.70476795139</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>4586808</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4586708</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4586708</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>46084.70482167824</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>4586708</v>
+      </c>
+      <c r="C18" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" t="n">
+        <v>36</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4586644</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4586644</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="n">
+        <v>46084.70494974537</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>4586644</v>
+      </c>
+      <c r="C19" t="n">
+        <v>100</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4586544</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4586544</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>46084.70502033565</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>4586544</v>
+      </c>
+      <c r="C20" t="n">
+        <v>100</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4586444</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4586444</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>46084.7051069213</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>4586444</v>
+      </c>
+      <c r="C21" t="n">
+        <v>100</v>
+      </c>
+      <c r="D21" t="n">
+        <v>60</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4586404</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4586404</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>46084.70523432871</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4586404</v>
+      </c>
+      <c r="C22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4586304</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4586304</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>46084.7053240625</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>4586304</v>
+      </c>
+      <c r="C23" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4586204</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4586204</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="n">
+        <v>46084.70542671296</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4586204</v>
+      </c>
+      <c r="C24" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4586104</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4586104</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="n">
+        <v>46084.70551292824</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>4586104</v>
+      </c>
+      <c r="C25" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4586004</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4586004</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="n">
+        <v>46084.70560280092</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4585904</v>
+      </c>
+      <c r="C26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4585804</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4585804</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="n">
+        <v>46084.73475758579</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>4585804</v>
+      </c>
+      <c r="C27" t="n">
+        <v>100</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4585704</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4585704</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="n">
+        <v>46084.73505033655</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>4585704</v>
+      </c>
+      <c r="C28" t="n">
+        <v>100</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4585604</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4585780</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-176</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="n">
+        <v>46084.73534017232</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4585780</v>
+      </c>
+      <c r="C29" t="n">
+        <v>100</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4585680</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4585680</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="n">
+        <v>46084.7356310456</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4585680</v>
+      </c>
+      <c r="C30" t="n">
+        <v>100</v>
+      </c>
+      <c r="D30" t="n">
+        <v>80</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4585660</v>
+      </c>
+      <c r="F30" t="n">
+        <v>4585660</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="n">
+        <v>46084.73593397777</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>4585660</v>
+      </c>
+      <c r="C31" t="n">
+        <v>100</v>
+      </c>
+      <c r="D31" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4585580</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4585580</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="n">
+        <v>46084.73622385836</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Setting the delay until suitable
</commit_message>
<xml_diff>
--- a/Slot_result.xlsx
+++ b/Slot_result.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,22 +471,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>9202518</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9202268</v>
+        <v>-200</v>
       </c>
       <c r="F2" t="n">
-        <v>4613779</v>
+        <v>349300</v>
       </c>
       <c r="G2" t="n">
-        <v>4588489</v>
+        <v>-349500</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>46084.60565237269</v>
+        <v>46085.48237882463</v>
       </c>
     </row>
     <row r="3">
@@ -502,19 +502,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>4613779</v>
+        <v>349300</v>
       </c>
       <c r="C3" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>4613529</v>
+        <v>349100</v>
       </c>
       <c r="F3" t="n">
-        <v>4613529</v>
+        <v>349100</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>46084.60593363426</v>
+        <v>46085.48250736086</v>
       </c>
     </row>
     <row r="4">
@@ -533,19 +533,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4613529</v>
+        <v>349100</v>
       </c>
       <c r="C4" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D4" t="n">
-        <v>1785</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>4615064</v>
+        <v>348900</v>
       </c>
       <c r="F4" t="n">
-        <v>4615064</v>
+        <v>348900</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>46084.6061349537</v>
+        <v>46085.48263771184</v>
       </c>
     </row>
     <row r="5">
@@ -564,30 +564,30 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>9202518</v>
+        <v>348900</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>9202518</v>
+        <v>348700</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>348700</v>
       </c>
       <c r="G5" t="n">
-        <v>9202518</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>46084.60917446759</v>
+        <v>46085.48276611464</v>
       </c>
     </row>
     <row r="6">
@@ -595,19 +595,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4615064</v>
+        <v>348700</v>
       </c>
       <c r="C6" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>4614814</v>
+        <v>348500</v>
       </c>
       <c r="F6" t="n">
-        <v>4614814</v>
+        <v>348500</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="I6" s="1" t="n">
-        <v>46084.60930747478</v>
+        <v>46085.48289443157</v>
       </c>
     </row>
     <row r="7">
@@ -626,30 +626,30 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>4614814</v>
+        <v>348500</v>
       </c>
       <c r="C7" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D7" t="n">
-        <v>140</v>
+        <v>2464</v>
       </c>
       <c r="E7" t="n">
-        <v>4614704</v>
+        <v>350764</v>
       </c>
       <c r="F7" t="n">
-        <v>4614564</v>
+        <v>350764</v>
       </c>
       <c r="G7" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I7" s="1" t="n">
-        <v>46084.60936990834</v>
+        <v>46085.48302450273</v>
       </c>
     </row>
     <row r="8">
@@ -657,30 +657,30 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>4614564</v>
+        <v>350764</v>
       </c>
       <c r="C8" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D8" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="E8" t="n">
-        <v>4614874</v>
+        <v>350684</v>
       </c>
       <c r="F8" t="n">
-        <v>4615124</v>
+        <v>350684</v>
       </c>
       <c r="G8" t="n">
-        <v>-250</v>
+        <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I8" s="1" t="n">
-        <v>46084.60942412478</v>
+        <v>46085.48315296327</v>
       </c>
     </row>
     <row r="9">
@@ -688,30 +688,278 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>4615124</v>
+        <v>350684</v>
       </c>
       <c r="C9" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="D9" t="n">
-        <v>1120</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>4615994</v>
+        <v>350484</v>
       </c>
       <c r="F9" t="n">
-        <v>4615684</v>
+        <v>350484</v>
       </c>
       <c r="G9" t="n">
-        <v>310</v>
+        <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>46085.48328111992</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>350484</v>
+      </c>
+      <c r="C10" t="n">
+        <v>200</v>
+      </c>
+      <c r="D10" t="n">
+        <v>120</v>
+      </c>
+      <c r="E10" t="n">
+        <v>350404</v>
+      </c>
+      <c r="F10" t="n">
+        <v>350404</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>46085.48340988783</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>350404</v>
+      </c>
+      <c r="C11" t="n">
+        <v>200</v>
+      </c>
+      <c r="D11" t="n">
+        <v>80</v>
+      </c>
+      <c r="E11" t="n">
+        <v>350284</v>
+      </c>
+      <c r="F11" t="n">
+        <v>350284</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>46085.48354127203</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>350284</v>
+      </c>
+      <c r="C12" t="n">
+        <v>200</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>350084</v>
+      </c>
+      <c r="F12" t="n">
+        <v>350084</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>46085.4836702378</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>350084</v>
+      </c>
+      <c r="C13" t="n">
+        <v>200</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>349884</v>
+      </c>
+      <c r="F13" t="n">
+        <v>349884</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="n">
+        <v>46085.48379847141</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>349884</v>
+      </c>
+      <c r="C14" t="n">
+        <v>200</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>349684</v>
+      </c>
+      <c r="F14" t="n">
+        <v>349684</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="n">
+        <v>46085.48392726513</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>349684</v>
+      </c>
+      <c r="C15" t="n">
+        <v>200</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>349484</v>
+      </c>
+      <c r="F15" t="n">
+        <v>349580</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-96</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Incorrect</t>
         </is>
       </c>
-      <c r="I9" s="1" t="n">
-        <v>46084.60977122879</v>
+      <c r="I15" s="1" t="n">
+        <v>46085.48405677947</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>349580</v>
+      </c>
+      <c r="C16" t="n">
+        <v>200</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>349380</v>
+      </c>
+      <c r="F16" t="n">
+        <v>349380</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="n">
+        <v>46085.48418875229</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>349380</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>349380</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>349380</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="n">
+        <v>46085.48506801661</v>
       </c>
     </row>
   </sheetData>

</xml_diff>